<commit_message>
Update bridesmaid names: Olivia Leon Vitervo, Yamilet Macias
Applied in both guest-codes.json (RSVP lookup) and the Guest List /
Guest Codes tabs of WEDDING_GUEST_LIST.xlsx. Invite codes unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019j1gnnKAkiNuhvSJorzwuc
</commit_message>
<xml_diff>
--- a/WEDDING_GUEST_LIST.xlsx
+++ b/WEDDING_GUEST_LIST.xlsx
@@ -631,10 +631,10 @@
     <t xml:space="preserve">Charnae</t>
   </si>
   <si>
-    <t xml:space="preserve">Olivia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yamilette</t>
+    <t xml:space="preserve">Olivia Leon Vitervo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yamilet Macias</t>
   </si>
   <si>
     <t xml:space="preserve">Kulsoom</t>

</xml_diff>